<commit_message>
Harden CRAMPS program language and generated artifacts
</commit_message>
<xml_diff>
--- a/spreadsheets/CRAMPS_Governance_Master.xlsx
+++ b/spreadsheets/CRAMPS_Governance_Master.xlsx
@@ -2,26 +2,26 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdd01e579565a463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="Rb0108151d58f4c3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="R0089b7e95a924028"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R39268fcdd04f4e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Catalog" sheetId="5" r:id="R3f872e6a1bb145a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assurance Claims" sheetId="6" r:id="R1d51d8218a8445b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supervisor Questions" sheetId="7" r:id="R281402ccece942da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Batteries" sheetId="8" r:id="R476bdd15df9243a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Scaffold" sheetId="9" r:id="R84f90a2869484c18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Registers" sheetId="10" r:id="Ra7307d9901a14406"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Controls" sheetId="11" r:id="R2d83b04ab859457f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training Paths" sheetId="12" r:id="R601188736fa94e0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework Patterns" sheetId="13" r:id="Rba2f121d274c467b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trust States" sheetId="14" r:id="Rcef51f5c5d804cbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reliance Levels" sheetId="15" r:id="Rc4eb1db60b754350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trust Checkpoints" sheetId="16" r:id="R4231cc4ba1944b84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPA Log" sheetId="17" r:id="Rbb1943c580bf4234"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="18" r:id="Rc3954d99ab6e4f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="19" r:id="R8517cc97a8804f3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="20" r:id="Rf715317f741d4671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8c5c19492f3c4cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="R79da42f988114511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="Rb3aea468edad4a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R70a7d2ec960e4510"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Catalog" sheetId="5" r:id="R5a81fd772cee4332"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assurance Claims" sheetId="6" r:id="R9d630098cdf548aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supervisor Questions" sheetId="7" r:id="R40d66da17c3548b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Batteries" sheetId="8" r:id="R803cc4bf51834cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Scaffold" sheetId="9" r:id="R99dd8ee6c08b4877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Registers" sheetId="10" r:id="R4f14c132e50549de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Controls" sheetId="11" r:id="Rfbfc4e8b7151416c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training Paths" sheetId="12" r:id="Rcfe57d7b720b42f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework Patterns" sheetId="13" r:id="R48b47c8a536c45bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trust States" sheetId="14" r:id="R1a92cff589bf4fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reliance Levels" sheetId="15" r:id="R6cdd7c4aded44951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trust Checkpoints" sheetId="16" r:id="R49b265bf1d7b4fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPA Log" sheetId="17" r:id="R63f55818414643a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure Modes" sheetId="18" r:id="Rd951ccbb24df4713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="19" r:id="R0a702a9aca6b46ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="20" r:id="Rf90f0c0e0b2e45b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,7 +221,7 @@
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Coordinate-resolved weak-signal recurrence governance</x:v>
+        <x:v>Coordinate-resolved weak-evidence inspection and recurrence governance</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1121,13 +1121,13 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Gotcha</x:v>
+        <x:v>Failure mode</x:v>
       </x:c>
       <x:c r="B1" t="str">
         <x:v>Symptom</x:v>
       </x:c>
       <x:c r="C1" t="str">
-        <x:v>Fast sanity check</x:v>
+        <x:v>Fast check</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1353,7 +1353,7 @@
         <x:v>Null Examples</x:v>
       </x:c>
       <x:c r="F1" t="str">
-        <x:v>Primary Gotchas</x:v>
+        <x:v>Primary Failure Modes</x:v>
       </x:c>
       <x:c r="G1" t="str">
         <x:v>Standards</x:v>
@@ -1720,13 +1720,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Gotchas</x:v>
+        <x:v>Failure Modes</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Fast failure-mode checks and stop signs</x:v>
+        <x:v>Fast checks, stop signs, and quarantine triggers</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>gotcha guide, field printouts</x:v>
+        <x:v>failure-mode guide, field printouts</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1927,7 +1927,7 @@
         <x:v>G3 Row Integrity</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>raw rows, source trace, extraction confidence, review status, quarantine log</x:v>
+        <x:v>raw signal rows, source trace, extraction confidence, review status, quarantine log</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>Before normalization closeout</x:v>
@@ -2426,7 +2426,7 @@
         <x:v>raw/normalized split, transform registry</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>hidden conversion created cluster</x:v>
+        <x:v>hidden conversion created apparent recurrence</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2454,7 +2454,7 @@
         <x:v>bias table, missing-evidence memo</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>reporting bias explains cluster</x:v>
+        <x:v>reporting bias explains recurrence</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2713,13 +2713,13 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Synthetic planted cluster</x:v>
+        <x:v>Controlled recurrence injection</x:v>
       </x:c>
       <x:c r="C3" t="str">
         <x:v>Known recurrence is injected</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>Detects planted recurrence under registered statistic</x:v>
+        <x:v>Recovers controlled recurrence under registered statistic</x:v>
       </x:c>
       <x:c r="E3" t="str"/>
       <x:c r="F3" t="str"/>
@@ -2846,7 +2846,7 @@
         <x:v>03_extraction</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>raw rows and extraction review</x:v>
+        <x:v>raw signal rows and extraction review</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>anomaly_rows_raw.csv; extraction_notes.md</x:v>

</xml_diff>